<commit_message>
title + some details notes
</commit_message>
<xml_diff>
--- a/timesheets/Dominik.xlsx
+++ b/timesheets/Dominik.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\domin\Documents\GitHub\wu_dslab_infrared-city\timesheets\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/130a09d975ce9163/Documents/GitHub/wu_dslab_infrared-city/timesheets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E92B7C3A-FE90-4EDA-962A-4FB2D778A384}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="11" documentId="13_ncr:1_{E92B7C3A-FE90-4EDA-962A-4FB2D778A384}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{980B0FF3-74AE-4A8B-B0D0-1496C902965B}"/>
   <bookViews>
-    <workbookView xWindow="40680" yWindow="2280" windowWidth="28800" windowHeight="15910" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-93" yWindow="-93" windowWidth="25786" windowHeight="15466" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="10">
   <si>
     <t>Date</t>
   </si>
@@ -57,6 +57,15 @@
   </si>
   <si>
     <t>Template project proposal, meetings + communication</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> </t>
+  </si>
+  <si>
+    <t>meetings</t>
+  </si>
+  <si>
+    <t>create second teams and regular meetings and communication</t>
   </si>
 </sst>
 </file>
@@ -375,15 +384,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H4"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:H72"/>
+  <sheetFormatPr defaultRowHeight="14.35" x14ac:dyDescent="0.5"/>
   <cols>
-    <col min="1" max="1" width="13.26953125" customWidth="1"/>
-    <col min="2" max="2" width="59.26953125" customWidth="1"/>
-    <col min="8" max="8" width="9.90625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.29296875" customWidth="1"/>
+    <col min="2" max="2" width="59.29296875" customWidth="1"/>
+    <col min="8" max="8" width="9.87890625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.5">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -397,7 +406,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.5">
       <c r="A2" s="1">
         <v>46090</v>
       </c>
@@ -409,10 +418,10 @@
       </c>
       <c r="H2">
         <f>SUM(C:C)</f>
-        <v>7.5</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
+        <v>9.75</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.5">
       <c r="A3" s="1">
         <v>46090</v>
       </c>
@@ -423,7 +432,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.5">
       <c r="A4" s="1">
         <v>46091</v>
       </c>
@@ -432,6 +441,358 @@
       </c>
       <c r="C4">
         <v>1.5</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.5">
+      <c r="A5" s="1">
+        <v>46094</v>
+      </c>
+      <c r="B5" t="s">
+        <v>8</v>
+      </c>
+      <c r="C5">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.5">
+      <c r="A6" s="1">
+        <v>46094</v>
+      </c>
+      <c r="B6" t="s">
+        <v>9</v>
+      </c>
+      <c r="C6">
+        <v>0.75</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.5">
+      <c r="A7" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.5">
+      <c r="A8" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.5">
+      <c r="A9" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.5">
+      <c r="A10" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.5">
+      <c r="A11" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.5">
+      <c r="A12" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.5">
+      <c r="A13" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.5">
+      <c r="A14" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.5">
+      <c r="A15" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.5">
+      <c r="A16" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.5">
+      <c r="A17" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.5">
+      <c r="A18" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1" x14ac:dyDescent="0.5">
+      <c r="A19" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1" x14ac:dyDescent="0.5">
+      <c r="A20" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="21" spans="1:1" x14ac:dyDescent="0.5">
+      <c r="A21" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1" x14ac:dyDescent="0.5">
+      <c r="A22" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="23" spans="1:1" x14ac:dyDescent="0.5">
+      <c r="A23" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="24" spans="1:1" x14ac:dyDescent="0.5">
+      <c r="A24" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="25" spans="1:1" x14ac:dyDescent="0.5">
+      <c r="A25" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="26" spans="1:1" x14ac:dyDescent="0.5">
+      <c r="A26" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="27" spans="1:1" x14ac:dyDescent="0.5">
+      <c r="A27" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="28" spans="1:1" x14ac:dyDescent="0.5">
+      <c r="A28" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="29" spans="1:1" x14ac:dyDescent="0.5">
+      <c r="A29" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="30" spans="1:1" x14ac:dyDescent="0.5">
+      <c r="A30" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="31" spans="1:1" x14ac:dyDescent="0.5">
+      <c r="A31" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="32" spans="1:1" x14ac:dyDescent="0.5">
+      <c r="A32" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="33" spans="1:1" x14ac:dyDescent="0.5">
+      <c r="A33" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="34" spans="1:1" x14ac:dyDescent="0.5">
+      <c r="A34" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="35" spans="1:1" x14ac:dyDescent="0.5">
+      <c r="A35" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="36" spans="1:1" x14ac:dyDescent="0.5">
+      <c r="A36" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="37" spans="1:1" x14ac:dyDescent="0.5">
+      <c r="A37" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="38" spans="1:1" x14ac:dyDescent="0.5">
+      <c r="A38" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="39" spans="1:1" x14ac:dyDescent="0.5">
+      <c r="A39" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="40" spans="1:1" x14ac:dyDescent="0.5">
+      <c r="A40" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="41" spans="1:1" x14ac:dyDescent="0.5">
+      <c r="A41" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="42" spans="1:1" x14ac:dyDescent="0.5">
+      <c r="A42" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="43" spans="1:1" x14ac:dyDescent="0.5">
+      <c r="A43" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="44" spans="1:1" x14ac:dyDescent="0.5">
+      <c r="A44" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="45" spans="1:1" x14ac:dyDescent="0.5">
+      <c r="A45" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="46" spans="1:1" x14ac:dyDescent="0.5">
+      <c r="A46" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="47" spans="1:1" x14ac:dyDescent="0.5">
+      <c r="A47" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="48" spans="1:1" x14ac:dyDescent="0.5">
+      <c r="A48" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="49" spans="1:1" x14ac:dyDescent="0.5">
+      <c r="A49" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="50" spans="1:1" x14ac:dyDescent="0.5">
+      <c r="A50" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="51" spans="1:1" x14ac:dyDescent="0.5">
+      <c r="A51" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="52" spans="1:1" x14ac:dyDescent="0.5">
+      <c r="A52" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="53" spans="1:1" x14ac:dyDescent="0.5">
+      <c r="A53" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="54" spans="1:1" x14ac:dyDescent="0.5">
+      <c r="A54" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="55" spans="1:1" x14ac:dyDescent="0.5">
+      <c r="A55" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="56" spans="1:1" x14ac:dyDescent="0.5">
+      <c r="A56" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="57" spans="1:1" x14ac:dyDescent="0.5">
+      <c r="A57" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="58" spans="1:1" x14ac:dyDescent="0.5">
+      <c r="A58" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="59" spans="1:1" x14ac:dyDescent="0.5">
+      <c r="A59" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="60" spans="1:1" x14ac:dyDescent="0.5">
+      <c r="A60" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="61" spans="1:1" x14ac:dyDescent="0.5">
+      <c r="A61" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="62" spans="1:1" x14ac:dyDescent="0.5">
+      <c r="A62" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="63" spans="1:1" x14ac:dyDescent="0.5">
+      <c r="A63" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="64" spans="1:1" x14ac:dyDescent="0.5">
+      <c r="A64" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="65" spans="1:1" x14ac:dyDescent="0.5">
+      <c r="A65" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="66" spans="1:1" x14ac:dyDescent="0.5">
+      <c r="A66" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="67" spans="1:1" x14ac:dyDescent="0.5">
+      <c r="A67" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="68" spans="1:1" x14ac:dyDescent="0.5">
+      <c r="A68" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="69" spans="1:1" x14ac:dyDescent="0.5">
+      <c r="A69" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="70" spans="1:1" x14ac:dyDescent="0.5">
+      <c r="A70" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="71" spans="1:1" x14ac:dyDescent="0.5">
+      <c r="A71" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="72" spans="1:1" x14ac:dyDescent="0.5">
+      <c r="A72" s="1" t="s">
+        <v>7</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add urban tree literature and update project plan
Add two new literature PDFs and BibTeX entries for recent urban tree classification papers, and include them in the project plan. Files added: deliverables/1. project plan/literature/IMPROVING URBAN TREE SPECIES CLASSIFICATION WITH HIGH RESOLUTION.pdf and Object-based classification of urban plant species from very high-resolution satellite imagery .pdf. Updated deliverables/1. project plan/literatur.bib with entries sicard2023object and wenger2024improving, referenced from deliverables/1. project plan/project_plan.tex (and the regenerated project_plan.pdf). Also updated timesheets/Dominik.xlsx.
</commit_message>
<xml_diff>
--- a/timesheets/Dominik.xlsx
+++ b/timesheets/Dominik.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/130a09d975ce9163/Documents/GitHub/wu_dslab_infrared-city/timesheets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="14" documentId="13_ncr:1_{E92B7C3A-FE90-4EDA-962A-4FB2D778A384}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1FC3E6A1-1B84-4F4E-BE6A-F569D4E8A3DD}"/>
+  <xr:revisionPtr revIDLastSave="17" documentId="13_ncr:1_{E92B7C3A-FE90-4EDA-962A-4FB2D778A384}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FC6623AB-50FD-4951-9CD5-C22FD4874931}"/>
   <bookViews>
     <workbookView xWindow="-93" yWindow="-93" windowWidth="25786" windowHeight="15466" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="12">
   <si>
     <t>Date</t>
   </si>
@@ -69,6 +69,9 @@
   </si>
   <si>
     <t>write first version of communication and teams in project proposal</t>
+  </si>
+  <si>
+    <t>add bibtex, rewrite literature, search new literature</t>
   </si>
 </sst>
 </file>
@@ -425,7 +428,7 @@
       </c>
       <c r="H2">
         <f>SUM(C:C)</f>
-        <v>11.25</v>
+        <v>12</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.5">
@@ -484,8 +487,14 @@
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.5">
-      <c r="A8" s="1" t="s">
-        <v>7</v>
+      <c r="A8" s="1">
+        <v>46096</v>
+      </c>
+      <c r="B8" t="s">
+        <v>11</v>
+      </c>
+      <c r="C8">
+        <v>0.75</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.5">

</xml_diff>

<commit_message>
report and slides template
</commit_message>
<xml_diff>
--- a/timesheets/Dominik.xlsx
+++ b/timesheets/Dominik.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\domin\Documents\GitHub\wu_dslab_infrared-city\timesheets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3594B57B-80C9-4081-9B4D-BCC4A894BAA6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{78F99C9B-D208-495A-99DA-5DA4B8F6C1A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3420" yWindow="3420" windowWidth="28800" windowHeight="15370" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="41160" yWindow="1310" windowWidth="28800" windowHeight="15370" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="25">
   <si>
     <t>Date</t>
   </si>
@@ -108,6 +108,9 @@
   </si>
   <si>
     <t>start finding of dates for sparring meeting</t>
+  </si>
+  <si>
+    <t>think about chapters in report, create template for report and slides</t>
   </si>
 </sst>
 </file>
@@ -460,7 +463,7 @@
       </c>
       <c r="H2">
         <f>SUM(C:C)</f>
-        <v>28.25</v>
+        <v>31.25</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.35">
@@ -662,8 +665,14 @@
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A21" s="1" t="s">
-        <v>7</v>
+      <c r="A21" s="1">
+        <v>46118</v>
+      </c>
+      <c r="B21" t="s">
+        <v>24</v>
+      </c>
+      <c r="C21">
+        <v>3</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
replace slides with template from wu
</commit_message>
<xml_diff>
--- a/timesheets/Dominik.xlsx
+++ b/timesheets/Dominik.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\domin\Documents\GitHub\wu_dslab_infrared-city\timesheets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{717358F8-3261-4D7C-86AA-A3BB65ED0115}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8B070A9E-05AD-47B3-B1FD-B4C4D920F1DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="41160" yWindow="1310" windowWidth="28800" windowHeight="15370" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="5530" yWindow="1990" windowWidth="28800" windowHeight="15370" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="32">
   <si>
     <t>Date</t>
   </si>
@@ -114,6 +114,24 @@
   </si>
   <si>
     <t>subtickets and planning of report and presentation + prepare agenda for tomorrow</t>
+  </si>
+  <si>
+    <t>weekly meeting in team + direct followup</t>
+  </si>
+  <si>
+    <t>Need</t>
+  </si>
+  <si>
+    <t>Open Weeks</t>
+  </si>
+  <si>
+    <t>End Datum</t>
+  </si>
+  <si>
+    <t>Need Hours</t>
+  </si>
+  <si>
+    <t>Need per week</t>
   </si>
 </sst>
 </file>
@@ -149,9 +167,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="16" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -432,15 +452,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H72"/>
+  <dimension ref="A1:R72"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="13.26953125" customWidth="1"/>
     <col min="2" max="2" width="71.54296875" customWidth="1"/>
     <col min="8" max="8" width="9.90625" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="13.36328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -453,8 +474,14 @@
       <c r="H1" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="Q1" t="s">
+        <v>29</v>
+      </c>
+      <c r="R1" s="2">
+        <v>46201</v>
+      </c>
+    </row>
+    <row r="2" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A2" s="1">
         <v>46090</v>
       </c>
@@ -466,10 +493,16 @@
       </c>
       <c r="H2">
         <f>SUM(C:C)</f>
-        <v>32.25</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
+        <v>34.75</v>
+      </c>
+      <c r="Q2" t="s">
+        <v>27</v>
+      </c>
+      <c r="R2">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="3" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A3" s="1">
         <v>46090</v>
       </c>
@@ -479,8 +512,15 @@
       <c r="C3">
         <v>2</v>
       </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="Q3" t="s">
+        <v>28</v>
+      </c>
+      <c r="R3" s="3">
+        <f ca="1">(R1 - TODAY()) / 7</f>
+        <v>11.428571428571429</v>
+      </c>
+    </row>
+    <row r="4" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A4" s="1">
         <v>46091</v>
       </c>
@@ -491,7 +531,7 @@
         <v>1.5</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A5" s="1">
         <v>46094</v>
       </c>
@@ -501,8 +541,15 @@
       <c r="C5">
         <v>1.5</v>
       </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="Q5" t="s">
+        <v>30</v>
+      </c>
+      <c r="R5">
+        <f>R2-H2</f>
+        <v>85.25</v>
+      </c>
+    </row>
+    <row r="6" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A6" s="1">
         <v>46094</v>
       </c>
@@ -512,8 +559,15 @@
       <c r="C6">
         <v>0.75</v>
       </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="Q6" t="s">
+        <v>31</v>
+      </c>
+      <c r="R6">
+        <f ca="1">R5/R3</f>
+        <v>7.4593749999999996</v>
+      </c>
+    </row>
+    <row r="7" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A7" s="1">
         <v>46095</v>
       </c>
@@ -524,7 +578,7 @@
         <v>1.5</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A8" s="1">
         <v>46096</v>
       </c>
@@ -535,7 +589,7 @@
         <v>0.75</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A9" s="1">
         <v>46096</v>
       </c>
@@ -546,7 +600,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A10" s="1">
         <v>46097</v>
       </c>
@@ -557,7 +611,7 @@
         <v>0.25</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A11" s="1">
         <v>46097</v>
       </c>
@@ -568,7 +622,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A12" s="1">
         <v>46099</v>
       </c>
@@ -579,7 +633,7 @@
         <v>0.25</v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A13" s="1">
         <v>46100</v>
       </c>
@@ -590,7 +644,7 @@
         <v>1.25</v>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A14" s="1">
         <v>46102</v>
       </c>
@@ -601,7 +655,7 @@
         <v>0.25</v>
       </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A15" s="1">
         <v>46104</v>
       </c>
@@ -612,7 +666,7 @@
         <v>0.75</v>
       </c>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A16" s="1">
         <v>46106</v>
       </c>
@@ -690,8 +744,14 @@
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A23" s="1" t="s">
-        <v>7</v>
+      <c r="A23" s="1">
+        <v>46121</v>
+      </c>
+      <c r="B23" t="s">
+        <v>26</v>
+      </c>
+      <c r="C23">
+        <v>2.5</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.35">
@@ -941,5 +1001,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>